<commit_message>
fix: simplify comment upload template
</commit_message>
<xml_diff>
--- a/templates/event-voc/comment_upload_template.xlsx
+++ b/templates/event-voc/comment_upload_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="VOC看事件-评论上传模板" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VOC看事件-评论上传模板" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -450,8 +450,6 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -492,32 +490,22 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>回复层级</t>
+          <t>评论正文</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>评论正文</t>
+          <t>评论发布时间</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>评论发布时间</t>
+          <t>评论点赞数</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>评论点赞数</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
           <t>评论回复数</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>评论原始链接</t>
         </is>
       </c>
     </row>
@@ -549,19 +537,19 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>必填</t>
@@ -569,20 +557,10 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>必填</t>
+          <t>选填</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>选填</t>
         </is>
@@ -616,7 +594,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>评论者昵称</t>
+          <t>评论者昵称，缺失时按未知用户处理</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -626,32 +604,22 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>空值按1处理</t>
+          <t>VOC原文</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>VOC原文</t>
+          <t>YYYY-MM-DD HH:MM:SS</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD HH:MM:SS</t>
+          <t>空值按0处理</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>空值按0处理</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>空值按0处理</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>评论链接，可为空</t>
         </is>
       </c>
     </row>
@@ -675,29 +643,21 @@
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="n">
-        <v>1</v>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>这个价格如果有置换补贴就很香，想看看配置差异。</t>
+        </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>这个价格如果有置换补贴就很香，想看看配置差异。</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
           <t>2026-05-01 21:10:00</t>
         </is>
       </c>
+      <c r="J4" s="3" t="n">
+        <v>23</v>
+      </c>
       <c r="K4" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="L4" s="3" t="n">
         <v>4</v>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/comment/c-001</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add comment location field
</commit_message>
<xml_diff>
--- a/templates/event-voc/comment_upload_template.xlsx
+++ b/templates/event-voc/comment_upload_template.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -450,6 +450,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,35 +476,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>位置</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>评论作者ID</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>评论作者昵称</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>父评论ID</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>评论正文</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>评论发布时间</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>评论点赞数</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>评论回复数</t>
         </is>
@@ -547,20 +553,25 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>选填</t>
-        </is>
-      </c>
       <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>选填</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>选填</t>
         </is>
@@ -589,35 +600,40 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
+          <t>平台显示的位置/IP属地/城市，可为空</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
           <t>第一版不做跨平台用户识别</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>评论者昵称，缺失时按未知用户处理</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>回复关系，可为空</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>VOC原文</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>YYYY-MM-DD HH:MM:SS</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>空值按0处理</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>空值按0处理</t>
         </is>
@@ -636,27 +652,32 @@
           <t>抖音</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>喜欢旅行的小王</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>这个价格如果有置换补贴就很香，想看看配置差异。</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>2026-05-01 21:10:00</t>
         </is>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="K4" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="L4" s="3" t="n">
         <v>4</v>
       </c>
     </row>

</xml_diff>